<commit_message>
docs: add current state files for MeisaiTemplate, including codebase pointers and screenshots
</commit_message>
<xml_diff>
--- a/backend/feature_ApplicationRulesAndMeetingExpenses/db_tables_application_rules_meeting_expenses.xlsx
+++ b/backend/feature_ApplicationRulesAndMeetingExpenses/db_tables_application_rules_meeting_expenses.xlsx
@@ -27,7 +27,7 @@
     <definedName hidden="1" localSheetId="6" name="_xlnm._FilterDatabase">tm_keihi_kamoku!$A$1:$L$9</definedName>
     <definedName hidden="1" localSheetId="7" name="_xlnm._FilterDatabase">tr_meisai_sankasha!$A$1:$L$11</definedName>
     <definedName hidden="1" localSheetId="8" name="_xlnm._FilterDatabase">tm_sankasha_template!$A$1:$L$9</definedName>
-    <definedName hidden="1" localSheetId="9" name="_xlnm._FilterDatabase">tm_sankasha_template_shosai!$A$1:$L$9</definedName>
+    <definedName hidden="1" localSheetId="9" name="_xlnm._FilterDatabase">tm_sankasha_template_shosai!$A$1:$L$10</definedName>
     <definedName hidden="1" localSheetId="10" name="_xlnm._FilterDatabase">tm_meisai_template!$A$1:$K$5</definedName>
     <definedName hidden="1" localSheetId="11" name="_xlnm._FilterDatabase">tm_shutsuryoku_komoku_shurui!$A$1:$H$6</definedName>
     <definedName hidden="1" localSheetId="12" name="_xlnm._FilterDatabase">Relations!$A$1:$D$13</definedName>
@@ -190,7 +190,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1269" uniqueCount="337">
   <si>
     <t>Category</t>
   </si>
@@ -1035,49 +1035,34 @@
     <t>Sort order inside template</t>
   </si>
   <si>
+    <t>hojincode</t>
+  </si>
+  <si>
     <t>NULL</t>
   </si>
   <si>
-    <t>外貨の種類</t>
-  </si>
-  <si>
-    <t>gaika_shurui</t>
-  </si>
-  <si>
-    <t>Tên ngoại tệ</t>
-  </si>
-  <si>
-    <t>外貨金額</t>
-  </si>
-  <si>
-    <t>kingaku</t>
+    <t>外貨種類ID</t>
+  </si>
+  <si>
+    <t>gaika_shurui_id</t>
+  </si>
+  <si>
+    <t>varchar(29)</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>円換算金額</t>
+  </si>
+  <si>
+    <t>en_kansan_kingaku</t>
+  </si>
+  <si>
+    <t>để cho phép null giống kingaku đã tồn tại trong tm_meisai_template</t>
   </si>
   <si>
     <t>レート</t>
-  </si>
-  <si>
-    <t xml:space="preserve">	rate</t>
-  </si>
-  <si>
-    <t>外貨種類ID</t>
-  </si>
-  <si>
-    <t>gaika_shurui_id</t>
-  </si>
-  <si>
-    <t>varchar(29)</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>円換算金額</t>
-  </si>
-  <si>
-    <t>en_kansan_kingaku</t>
-  </si>
-  <si>
-    <t>để cho phép null giống kingaku đã tồn tại trong tm_meisai_template</t>
   </si>
   <si>
     <t xml:space="preserve">rate </t>
@@ -1263,7 +1248,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -1302,10 +1287,6 @@
     </font>
     <font>
       <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1409,7 +1390,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1449,23 +1430,17 @@
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="5" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
@@ -3305,7 +3280,11 @@
     <row r="9" ht="14.25" customHeight="1">
       <c r="J9" s="8"/>
     </row>
-    <row r="10" ht="14.25" customHeight="1"/>
+    <row r="10" ht="14.25" customHeight="1">
+      <c r="D10" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="B11" s="8" t="s">
         <v>184</v>
@@ -4340,7 +4319,7 @@
     <row r="999" ht="14.25" customHeight="1"/>
     <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$1:$L$9"/>
+  <autoFilter ref="$A$1:$L$10"/>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
@@ -4427,7 +4406,7 @@
         <v>70</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
@@ -4439,20 +4418,23 @@
       <c r="B3" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>282</v>
+      <c r="C3" s="3" t="s">
+        <v>283</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>124</v>
+        <v>284</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>285</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>284</v>
+      <c r="G3" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
@@ -4462,17 +4444,23 @@
       <c r="B4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>285</v>
+      <c r="C4" s="3" t="s">
+        <v>287</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>281</v>
+      <c r="I4" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -4482,17 +4470,23 @@
       <c r="B5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>287</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>288</v>
-      </c>
-      <c r="E5" s="8" t="s">
+      <c r="C5" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="I5" s="9" t="s">
-        <v>281</v>
+      <c r="G5" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="I5" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1"/>
@@ -4500,70 +4494,36 @@
     <row r="8" ht="14.25" customHeight="1"/>
     <row r="9" ht="14.25" customHeight="1"/>
     <row r="10" ht="14.25" customHeight="1">
-      <c r="C10" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>290</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>291</v>
-      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
       <c r="F10" s="14"/>
-      <c r="G10" s="3" t="s">
-        <v>292</v>
-      </c>
+      <c r="G10" s="3"/>
       <c r="H10" s="14"/>
-      <c r="I10" s="9" t="s">
-        <v>281</v>
-      </c>
+      <c r="I10" s="9"/>
       <c r="J10" s="14"/>
       <c r="K10" s="14"/>
     </row>
     <row r="11" ht="14.25" customHeight="1">
-      <c r="C11" s="15" t="s">
-        <v>293</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>67</v>
-      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
       <c r="F11" s="14"/>
-      <c r="G11" s="3" t="s">
-        <v>292</v>
-      </c>
+      <c r="G11" s="3"/>
       <c r="H11" s="14"/>
-      <c r="I11" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>295</v>
-      </c>
+      <c r="I11" s="9"/>
+      <c r="J11" s="3"/>
       <c r="K11" s="14"/>
     </row>
     <row r="12" ht="14.25" customHeight="1">
-      <c r="C12" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>67</v>
-      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
       <c r="F12" s="14"/>
-      <c r="G12" s="3" t="s">
-        <v>292</v>
-      </c>
+      <c r="G12" s="3"/>
       <c r="H12" s="14"/>
-      <c r="I12" s="16">
-        <v>1.0</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>297</v>
-      </c>
+      <c r="I12" s="13"/>
+      <c r="J12" s="3"/>
       <c r="K12" s="14"/>
     </row>
     <row r="13" ht="14.25" customHeight="1"/>
@@ -5598,448 +5558,448 @@
   </cols>
   <sheetData>
     <row r="1" ht="117.0" customHeight="1">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="15" t="s">
+        <v>293</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>294</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="F1" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="G1" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="H1" s="16" t="s">
         <v>298</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="I1" s="16" t="s">
         <v>299</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="J1" s="16" t="s">
         <v>300</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="K1" s="16" t="s">
         <v>301</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="L1" s="16" t="s">
         <v>302</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="M1" s="16" t="s">
         <v>303</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="N1" s="16" t="s">
         <v>304</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="O1" s="16" t="s">
         <v>305</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="P1" s="16" t="s">
         <v>306</v>
       </c>
-      <c r="L1" s="18" t="s">
+      <c r="Q1" s="16" t="s">
         <v>307</v>
       </c>
-      <c r="M1" s="18" t="s">
+      <c r="R1" s="16" t="s">
         <v>308</v>
       </c>
-      <c r="N1" s="18" t="s">
+      <c r="S1" s="16" t="s">
         <v>309</v>
       </c>
-      <c r="O1" s="18" t="s">
+      <c r="T1" s="16" t="s">
         <v>310</v>
       </c>
-      <c r="P1" s="18" t="s">
+      <c r="U1" s="16" t="s">
         <v>311</v>
       </c>
-      <c r="Q1" s="18" t="s">
+      <c r="V1" s="16" t="s">
         <v>312</v>
       </c>
-      <c r="R1" s="18" t="s">
+      <c r="W1" s="16" t="s">
         <v>313</v>
       </c>
-      <c r="S1" s="18" t="s">
+      <c r="X1" s="16" t="s">
         <v>314</v>
       </c>
-      <c r="T1" s="18" t="s">
-        <v>315</v>
-      </c>
-      <c r="U1" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="V1" s="18" t="s">
-        <v>317</v>
-      </c>
-      <c r="W1" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="X1" s="18" t="s">
-        <v>319</v>
-      </c>
-      <c r="Y1" s="19"/>
-      <c r="Z1" s="19"/>
+      <c r="Y1" s="17"/>
+      <c r="Z1" s="17"/>
     </row>
     <row r="2" ht="36.0" customHeight="1">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="21">
+      <c r="C2" s="19">
         <v>141.0</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="19" t="s">
         <v>269</v>
       </c>
-      <c r="E2" s="21">
+      <c r="E2" s="19">
         <v>1.0</v>
       </c>
-      <c r="F2" s="21">
+      <c r="F2" s="19">
         <v>0.0</v>
       </c>
-      <c r="G2" s="21">
+      <c r="G2" s="19">
         <v>0.0</v>
       </c>
-      <c r="H2" s="21">
+      <c r="H2" s="19">
         <v>1.0</v>
       </c>
-      <c r="I2" s="22">
+      <c r="I2" s="20">
         <v>0.0</v>
       </c>
-      <c r="J2" s="22">
+      <c r="J2" s="20">
         <v>0.0</v>
       </c>
-      <c r="K2" s="22">
+      <c r="K2" s="20">
         <v>2.0</v>
       </c>
-      <c r="L2" s="22">
+      <c r="L2" s="20">
         <v>0.0</v>
       </c>
-      <c r="M2" s="22">
+      <c r="M2" s="20">
         <v>1.0</v>
       </c>
-      <c r="N2" s="22">
+      <c r="N2" s="20">
         <v>0.0</v>
       </c>
-      <c r="O2" s="22">
+      <c r="O2" s="20">
         <v>0.0</v>
       </c>
-      <c r="P2" s="22">
+      <c r="P2" s="20">
         <v>0.0</v>
       </c>
-      <c r="Q2" s="22">
+      <c r="Q2" s="20">
         <v>0.0</v>
       </c>
-      <c r="R2" s="22">
+      <c r="R2" s="20">
         <v>1.0</v>
       </c>
-      <c r="S2" s="22">
+      <c r="S2" s="20">
         <v>0.0</v>
       </c>
-      <c r="T2" s="22">
+      <c r="T2" s="20">
         <v>0.0</v>
       </c>
-      <c r="U2" s="22">
+      <c r="U2" s="20">
         <v>0.0</v>
       </c>
-      <c r="V2" s="22">
+      <c r="V2" s="20">
         <v>0.0</v>
       </c>
-      <c r="W2" s="22">
+      <c r="W2" s="20">
         <v>0.0</v>
       </c>
-      <c r="X2" s="22">
+      <c r="X2" s="20">
         <v>920.0</v>
       </c>
     </row>
     <row r="3" ht="18.0" customHeight="1">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="21">
+      <c r="C3" s="19">
         <v>142.0</v>
       </c>
-      <c r="D3" s="21" t="s">
-        <v>320</v>
-      </c>
-      <c r="E3" s="21">
+      <c r="D3" s="19" t="s">
+        <v>315</v>
+      </c>
+      <c r="E3" s="19">
         <v>1.0</v>
       </c>
-      <c r="F3" s="21">
+      <c r="F3" s="19">
         <v>0.0</v>
       </c>
-      <c r="G3" s="21">
+      <c r="G3" s="19">
         <v>0.0</v>
       </c>
-      <c r="H3" s="21">
+      <c r="H3" s="19">
         <v>1.0</v>
       </c>
-      <c r="I3" s="22">
+      <c r="I3" s="20">
         <v>0.0</v>
       </c>
-      <c r="J3" s="22">
+      <c r="J3" s="20">
         <v>0.0</v>
       </c>
-      <c r="K3" s="22">
+      <c r="K3" s="20">
         <v>2.0</v>
       </c>
-      <c r="L3" s="22">
+      <c r="L3" s="20">
         <v>0.0</v>
       </c>
-      <c r="M3" s="22">
+      <c r="M3" s="20">
         <v>1.0</v>
       </c>
-      <c r="N3" s="22">
+      <c r="N3" s="20">
         <v>0.0</v>
       </c>
-      <c r="O3" s="22">
+      <c r="O3" s="20">
         <v>0.0</v>
       </c>
-      <c r="P3" s="22">
+      <c r="P3" s="20">
         <v>0.0</v>
       </c>
-      <c r="Q3" s="22">
+      <c r="Q3" s="20">
         <v>0.0</v>
       </c>
-      <c r="R3" s="22">
+      <c r="R3" s="20">
         <v>1.0</v>
       </c>
-      <c r="S3" s="22">
+      <c r="S3" s="20">
         <v>0.0</v>
       </c>
-      <c r="T3" s="22">
+      <c r="T3" s="20">
         <v>0.0</v>
       </c>
-      <c r="U3" s="22">
+      <c r="U3" s="20">
         <v>0.0</v>
       </c>
-      <c r="V3" s="22">
+      <c r="V3" s="20">
         <v>0.0</v>
       </c>
-      <c r="W3" s="22">
+      <c r="W3" s="20">
         <v>0.0</v>
       </c>
-      <c r="X3" s="22">
+      <c r="X3" s="20">
         <v>930.0</v>
       </c>
     </row>
     <row r="4" ht="18.0" customHeight="1">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="21">
+      <c r="C4" s="19">
         <v>143.0</v>
       </c>
-      <c r="D4" s="21" t="s">
-        <v>321</v>
-      </c>
-      <c r="E4" s="21">
+      <c r="D4" s="19" t="s">
+        <v>316</v>
+      </c>
+      <c r="E4" s="19">
         <v>1.0</v>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="19">
         <v>0.0</v>
       </c>
-      <c r="G4" s="21">
+      <c r="G4" s="19">
         <v>0.0</v>
       </c>
-      <c r="H4" s="21">
+      <c r="H4" s="19">
         <v>1.0</v>
       </c>
-      <c r="I4" s="22">
+      <c r="I4" s="20">
         <v>0.0</v>
       </c>
-      <c r="J4" s="22">
+      <c r="J4" s="20">
         <v>0.0</v>
       </c>
-      <c r="K4" s="22">
+      <c r="K4" s="20">
         <v>2.0</v>
       </c>
-      <c r="L4" s="22">
+      <c r="L4" s="20">
         <v>0.0</v>
       </c>
-      <c r="M4" s="22">
+      <c r="M4" s="20">
         <v>1.0</v>
       </c>
-      <c r="N4" s="22">
+      <c r="N4" s="20">
         <v>0.0</v>
       </c>
-      <c r="O4" s="22">
+      <c r="O4" s="20">
         <v>0.0</v>
       </c>
-      <c r="P4" s="22">
+      <c r="P4" s="20">
         <v>0.0</v>
       </c>
-      <c r="Q4" s="22">
+      <c r="Q4" s="20">
         <v>0.0</v>
       </c>
-      <c r="R4" s="22">
+      <c r="R4" s="20">
         <v>1.0</v>
       </c>
-      <c r="S4" s="22">
+      <c r="S4" s="20">
         <v>0.0</v>
       </c>
-      <c r="T4" s="22">
+      <c r="T4" s="20">
         <v>0.0</v>
       </c>
-      <c r="U4" s="22">
+      <c r="U4" s="20">
         <v>0.0</v>
       </c>
-      <c r="V4" s="22">
+      <c r="V4" s="20">
         <v>0.0</v>
       </c>
-      <c r="W4" s="22">
+      <c r="W4" s="20">
         <v>0.0</v>
       </c>
-      <c r="X4" s="22">
+      <c r="X4" s="20">
         <v>940.0</v>
       </c>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="21">
+      <c r="C5" s="19">
         <v>144.0</v>
       </c>
-      <c r="D5" s="21" t="s">
-        <v>322</v>
-      </c>
-      <c r="E5" s="21">
+      <c r="D5" s="19" t="s">
+        <v>317</v>
+      </c>
+      <c r="E5" s="19">
         <v>1.0</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="19">
         <v>0.0</v>
       </c>
-      <c r="G5" s="21">
+      <c r="G5" s="19">
         <v>0.0</v>
       </c>
-      <c r="H5" s="21">
+      <c r="H5" s="19">
         <v>1.0</v>
       </c>
-      <c r="I5" s="22">
+      <c r="I5" s="20">
         <v>0.0</v>
       </c>
-      <c r="J5" s="22">
+      <c r="J5" s="20">
         <v>0.0</v>
       </c>
-      <c r="K5" s="22">
+      <c r="K5" s="20">
         <v>2.0</v>
       </c>
-      <c r="L5" s="22">
+      <c r="L5" s="20">
         <v>0.0</v>
       </c>
-      <c r="M5" s="22">
+      <c r="M5" s="20">
         <v>1.0</v>
       </c>
-      <c r="N5" s="22">
+      <c r="N5" s="20">
         <v>0.0</v>
       </c>
-      <c r="O5" s="22">
+      <c r="O5" s="20">
         <v>0.0</v>
       </c>
-      <c r="P5" s="22">
+      <c r="P5" s="20">
         <v>0.0</v>
       </c>
-      <c r="Q5" s="22">
+      <c r="Q5" s="20">
         <v>0.0</v>
       </c>
-      <c r="R5" s="22">
+      <c r="R5" s="20">
         <v>1.0</v>
       </c>
-      <c r="S5" s="22">
+      <c r="S5" s="20">
         <v>0.0</v>
       </c>
-      <c r="T5" s="22">
+      <c r="T5" s="20">
         <v>0.0</v>
       </c>
-      <c r="U5" s="22">
+      <c r="U5" s="20">
         <v>0.0</v>
       </c>
-      <c r="V5" s="22">
+      <c r="V5" s="20">
         <v>0.0</v>
       </c>
-      <c r="W5" s="22">
+      <c r="W5" s="20">
         <v>0.0</v>
       </c>
-      <c r="X5" s="22">
+      <c r="X5" s="20">
         <v>950.0</v>
       </c>
     </row>
     <row r="6" ht="36.0" customHeight="1">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="19">
         <v>145.0</v>
       </c>
-      <c r="D6" s="20" t="s">
-        <v>323</v>
-      </c>
-      <c r="E6" s="21">
+      <c r="D6" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="E6" s="19">
         <v>1.0</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="19">
         <v>0.0</v>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="19">
         <v>0.0</v>
       </c>
-      <c r="H6" s="21">
+      <c r="H6" s="19">
         <v>1.0</v>
       </c>
-      <c r="I6" s="22">
+      <c r="I6" s="20">
         <v>0.0</v>
       </c>
-      <c r="J6" s="22">
+      <c r="J6" s="20">
         <v>0.0</v>
       </c>
-      <c r="K6" s="22">
+      <c r="K6" s="20">
         <v>2.0</v>
       </c>
-      <c r="L6" s="22">
+      <c r="L6" s="20">
         <v>0.0</v>
       </c>
-      <c r="M6" s="22">
+      <c r="M6" s="20">
         <v>1.0</v>
       </c>
-      <c r="N6" s="22">
+      <c r="N6" s="20">
         <v>0.0</v>
       </c>
-      <c r="O6" s="22">
+      <c r="O6" s="20">
         <v>0.0</v>
       </c>
-      <c r="P6" s="22">
+      <c r="P6" s="20">
         <v>0.0</v>
       </c>
-      <c r="Q6" s="22">
+      <c r="Q6" s="20">
         <v>0.0</v>
       </c>
-      <c r="R6" s="22">
+      <c r="R6" s="20">
         <v>1.0</v>
       </c>
-      <c r="S6" s="22">
+      <c r="S6" s="20">
         <v>0.0</v>
       </c>
-      <c r="T6" s="22">
+      <c r="T6" s="20">
         <v>0.0</v>
       </c>
-      <c r="U6" s="22">
+      <c r="U6" s="20">
         <v>0.0</v>
       </c>
-      <c r="V6" s="22">
+      <c r="V6" s="20">
         <v>0.0</v>
       </c>
-      <c r="W6" s="22">
+      <c r="W6" s="20">
         <v>0.0</v>
       </c>
-      <c r="X6" s="22">
+      <c r="X6" s="20">
         <v>960.0</v>
       </c>
     </row>
@@ -7061,13 +7021,13 @@
   <sheetData>
     <row r="1" ht="24.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -7078,13 +7038,13 @@
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
     </row>
     <row r="3" ht="18.0" customHeight="1">
@@ -7098,7 +7058,7 @@
         <v>12</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" ht="18.0" customHeight="1">
@@ -7106,13 +7066,13 @@
         <v>22</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
     </row>
     <row r="5" ht="18.0" customHeight="1">
@@ -7120,13 +7080,13 @@
         <v>25</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
     </row>
     <row r="6" ht="18.0" customHeight="1">
@@ -7134,13 +7094,13 @@
         <v>28</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
     </row>
     <row r="7" ht="18.0" customHeight="1">
@@ -7151,10 +7111,10 @@
         <v>199</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
     </row>
     <row r="8" ht="18.0" customHeight="1">
@@ -7168,7 +7128,7 @@
         <v>31</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="9" ht="18.0" customHeight="1">
@@ -7179,10 +7139,10 @@
         <v>254</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
     </row>
     <row r="10" ht="18.0" customHeight="1">
@@ -7193,10 +7153,10 @@
         <v>238</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
     </row>
     <row r="11" ht="18.0" customHeight="1">
@@ -7207,10 +7167,10 @@
         <v>254</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" ht="36.0" customHeight="1">
@@ -7224,7 +7184,7 @@
         <v>31</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13" ht="36.0" customHeight="1">
@@ -7232,13 +7192,13 @@
         <v>49</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>39</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1"/>
@@ -15390,7 +15350,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" ht="18.0" customHeight="1">
+    <row r="5">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
docs: add detailed design and finalized spec for KeihiKamoku extension, including API, DB schema, business rules, and validation logic
</commit_message>
<xml_diff>
--- a/backend/feature_ApplicationRulesAndMeetingExpenses/db_tables_application_rules_meeting_expenses.xlsx
+++ b/backend/feature_ApplicationRulesAndMeetingExpenses/db_tables_application_rules_meeting_expenses.xlsx
@@ -35,7 +35,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId17" roundtripDataChecksum="bYA+q8C9zZQNpEjt70Eyp5PvWHzEdK0R4zGZnY+fAA0="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId17" roundtripDataChecksum="jl0r7rq5dYXcNzcdwoWoFNo6n2q+yGnB/Up0po25af4="/>
     </ext>
   </extLst>
 </workbook>
@@ -47,6 +47,16 @@
     <author/>
   </authors>
   <commentList>
+    <comment authorId="0" ref="E21">
+      <text>
+        <t xml:space="preserve">======
+ID#AAAB7rVOAhs
+DucNA1    (2026-06-05 06:51:52)
+@hangvt@hblab.vn @anhntl@hblab.vn @duongnv2@hblab.vn theo expect mới do trường này được thực hiện search ở màn list nên mình sẽ thực hiện lưu thêm vào bảng tr_meisai_joho nhé. 
+Giải thích thêm: nếu trường này ko được search/sort thì sẽ không lưu vào db mà chỉ cần tính toán rồi trả ra thoi
+_Assigned to HangVT (Carrot_)_</t>
+      </text>
+    </comment>
     <comment authorId="0" ref="J9">
       <text>
         <t xml:space="preserve">======
@@ -66,7 +76,7 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mgOrlkLGPB/H9GXTcSoT44hVOE0qA=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7miU04G871omtswf+gh4LqHkQbV4bg=="/>
     </ext>
   </extLst>
 </comments>
@@ -105,7 +115,7 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7miyz8+fdk2vDmrIh5uFwZtCsRF0ag=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mihT4KygaXP2LcX2tVl9xUWB5CJPg=="/>
     </ext>
   </extLst>
 </comments>
@@ -136,7 +146,7 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mj+MY2+FYEpcOFsBILJsb6Q1mWl0Q=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mjFuprO1I6oaV4aFY8GZBoHHv9rCA=="/>
     </ext>
   </extLst>
 </comments>
@@ -183,14 +193,14 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mgYw2FQGg8x58bDjxwKzkma/pdeEQ=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mhDYPo7ukEM/UmKRXR1EG0K/Ky6OQ=="/>
     </ext>
   </extLst>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1269" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1269" uniqueCount="339">
   <si>
     <t>Category</t>
   </si>
@@ -828,6 +838,9 @@
     <t>hitori_atari_jogen_check_kubun</t>
   </si>
   <si>
+    <t>0: None 1: Error, 2: Alert</t>
+  </si>
+  <si>
     <t>一人当たり上限金額超過時のメッセージ</t>
   </si>
   <si>
@@ -967,6 +980,9 @@
   </si>
   <si>
     <t>(bổ sung spec mới)</t>
+  </si>
+  <si>
+    <t>hitori_atari_kingaku(số tiền/mỗi người) lưu thêm trong tr_meisai_joho</t>
   </si>
   <si>
     <t>参加者テンプレートID</t>
@@ -1390,7 +1406,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1421,11 +1437,14 @@
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -3019,13 +3038,13 @@
         <v>36</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>124</v>
@@ -3046,7 +3065,7 @@
         <v>127</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" ht="18.0" customHeight="1">
@@ -3057,13 +3076,13 @@
         <v>36</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>124</v>
@@ -3081,7 +3100,7 @@
         <v>70</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>70</v>
@@ -3095,13 +3114,13 @@
         <v>36</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>67</v>
@@ -3119,7 +3138,7 @@
         <v>70</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>70</v>
@@ -3133,19 +3152,19 @@
         <v>36</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>124</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>95</v>
@@ -3157,7 +3176,7 @@
         <v>70</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>70</v>
@@ -3171,19 +3190,19 @@
         <v>36</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>124</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>95</v>
@@ -3195,7 +3214,7 @@
         <v>70</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>70</v>
@@ -3209,13 +3228,13 @@
         <v>36</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>124</v>
@@ -3267,11 +3286,11 @@
       <c r="I8" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="J8" s="12" t="s">
-        <v>279</v>
+      <c r="J8" s="13" t="s">
+        <v>281</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>70</v>
@@ -3282,7 +3301,7 @@
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="D10" s="8" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -4388,10 +4407,10 @@
         <v>44</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>124</v>
@@ -4406,7 +4425,7 @@
         <v>70</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
@@ -4419,22 +4438,22 @@
         <v>44</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>125</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
@@ -4445,22 +4464,22 @@
         <v>44</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -4471,22 +4490,22 @@
         <v>44</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="I5" s="13">
+        <v>288</v>
+      </c>
+      <c r="I5" s="14">
         <v>1.0</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1"/>
@@ -4497,34 +4516,34 @@
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
-      <c r="F10" s="14"/>
+      <c r="F10" s="15"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="14"/>
+      <c r="H10" s="15"/>
       <c r="I10" s="9"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="14"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="14"/>
+      <c r="F11" s="15"/>
       <c r="G11" s="3"/>
-      <c r="H11" s="14"/>
+      <c r="H11" s="15"/>
       <c r="I11" s="9"/>
       <c r="J11" s="3"/>
-      <c r="K11" s="14"/>
+      <c r="K11" s="15"/>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
-      <c r="F12" s="14"/>
+      <c r="F12" s="15"/>
       <c r="G12" s="3"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="13"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="14"/>
       <c r="J12" s="3"/>
-      <c r="K12" s="14"/>
+      <c r="K12" s="15"/>
     </row>
     <row r="13" ht="14.25" customHeight="1"/>
     <row r="14" ht="14.25" customHeight="1"/>
@@ -5558,448 +5577,448 @@
   </cols>
   <sheetData>
     <row r="1" ht="117.0" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="C1" s="15" t="s">
-        <v>293</v>
-      </c>
-      <c r="D1" s="15" t="s">
-        <v>294</v>
-      </c>
-      <c r="E1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>295</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>296</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="E1" s="17" t="s">
         <v>297</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="F1" s="17" t="s">
         <v>298</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="G1" s="17" t="s">
         <v>299</v>
       </c>
-      <c r="J1" s="16" t="s">
+      <c r="H1" s="17" t="s">
         <v>300</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="I1" s="17" t="s">
         <v>301</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="J1" s="17" t="s">
         <v>302</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="K1" s="17" t="s">
         <v>303</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="L1" s="17" t="s">
         <v>304</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="M1" s="17" t="s">
         <v>305</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="N1" s="17" t="s">
         <v>306</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="O1" s="17" t="s">
         <v>307</v>
       </c>
-      <c r="R1" s="16" t="s">
+      <c r="P1" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="S1" s="16" t="s">
+      <c r="Q1" s="17" t="s">
         <v>309</v>
       </c>
-      <c r="T1" s="16" t="s">
+      <c r="R1" s="17" t="s">
         <v>310</v>
       </c>
-      <c r="U1" s="16" t="s">
+      <c r="S1" s="17" t="s">
         <v>311</v>
       </c>
-      <c r="V1" s="16" t="s">
+      <c r="T1" s="17" t="s">
         <v>312</v>
       </c>
-      <c r="W1" s="16" t="s">
+      <c r="U1" s="17" t="s">
         <v>313</v>
       </c>
-      <c r="X1" s="16" t="s">
+      <c r="V1" s="17" t="s">
         <v>314</v>
       </c>
-      <c r="Y1" s="17"/>
-      <c r="Z1" s="17"/>
+      <c r="W1" s="17" t="s">
+        <v>315</v>
+      </c>
+      <c r="X1" s="17" t="s">
+        <v>316</v>
+      </c>
+      <c r="Y1" s="18"/>
+      <c r="Z1" s="18"/>
     </row>
     <row r="2" ht="36.0" customHeight="1">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="19">
+      <c r="C2" s="20">
         <v>141.0</v>
       </c>
-      <c r="D2" s="19" t="s">
-        <v>269</v>
-      </c>
-      <c r="E2" s="19">
+      <c r="D2" s="20" t="s">
+        <v>271</v>
+      </c>
+      <c r="E2" s="20">
         <v>1.0</v>
       </c>
-      <c r="F2" s="19">
+      <c r="F2" s="20">
         <v>0.0</v>
       </c>
-      <c r="G2" s="19">
+      <c r="G2" s="20">
         <v>0.0</v>
       </c>
-      <c r="H2" s="19">
+      <c r="H2" s="20">
         <v>1.0</v>
       </c>
-      <c r="I2" s="20">
+      <c r="I2" s="21">
         <v>0.0</v>
       </c>
-      <c r="J2" s="20">
+      <c r="J2" s="21">
         <v>0.0</v>
       </c>
-      <c r="K2" s="20">
+      <c r="K2" s="21">
         <v>2.0</v>
       </c>
-      <c r="L2" s="20">
+      <c r="L2" s="21">
         <v>0.0</v>
       </c>
-      <c r="M2" s="20">
+      <c r="M2" s="21">
         <v>1.0</v>
       </c>
-      <c r="N2" s="20">
+      <c r="N2" s="21">
         <v>0.0</v>
       </c>
-      <c r="O2" s="20">
+      <c r="O2" s="21">
         <v>0.0</v>
       </c>
-      <c r="P2" s="20">
+      <c r="P2" s="21">
         <v>0.0</v>
       </c>
-      <c r="Q2" s="20">
+      <c r="Q2" s="21">
         <v>0.0</v>
       </c>
-      <c r="R2" s="20">
+      <c r="R2" s="21">
         <v>1.0</v>
       </c>
-      <c r="S2" s="20">
+      <c r="S2" s="21">
         <v>0.0</v>
       </c>
-      <c r="T2" s="20">
+      <c r="T2" s="21">
         <v>0.0</v>
       </c>
-      <c r="U2" s="20">
+      <c r="U2" s="21">
         <v>0.0</v>
       </c>
-      <c r="V2" s="20">
+      <c r="V2" s="21">
         <v>0.0</v>
       </c>
-      <c r="W2" s="20">
+      <c r="W2" s="21">
         <v>0.0</v>
       </c>
-      <c r="X2" s="20">
+      <c r="X2" s="21">
         <v>920.0</v>
       </c>
     </row>
     <row r="3" ht="18.0" customHeight="1">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="20">
         <v>142.0</v>
       </c>
-      <c r="D3" s="19" t="s">
-        <v>315</v>
-      </c>
-      <c r="E3" s="19">
+      <c r="D3" s="20" t="s">
+        <v>317</v>
+      </c>
+      <c r="E3" s="20">
         <v>1.0</v>
       </c>
-      <c r="F3" s="19">
+      <c r="F3" s="20">
         <v>0.0</v>
       </c>
-      <c r="G3" s="19">
+      <c r="G3" s="20">
         <v>0.0</v>
       </c>
-      <c r="H3" s="19">
+      <c r="H3" s="20">
         <v>1.0</v>
       </c>
-      <c r="I3" s="20">
+      <c r="I3" s="21">
         <v>0.0</v>
       </c>
-      <c r="J3" s="20">
+      <c r="J3" s="21">
         <v>0.0</v>
       </c>
-      <c r="K3" s="20">
+      <c r="K3" s="21">
         <v>2.0</v>
       </c>
-      <c r="L3" s="20">
+      <c r="L3" s="21">
         <v>0.0</v>
       </c>
-      <c r="M3" s="20">
+      <c r="M3" s="21">
         <v>1.0</v>
       </c>
-      <c r="N3" s="20">
+      <c r="N3" s="21">
         <v>0.0</v>
       </c>
-      <c r="O3" s="20">
+      <c r="O3" s="21">
         <v>0.0</v>
       </c>
-      <c r="P3" s="20">
+      <c r="P3" s="21">
         <v>0.0</v>
       </c>
-      <c r="Q3" s="20">
+      <c r="Q3" s="21">
         <v>0.0</v>
       </c>
-      <c r="R3" s="20">
+      <c r="R3" s="21">
         <v>1.0</v>
       </c>
-      <c r="S3" s="20">
+      <c r="S3" s="21">
         <v>0.0</v>
       </c>
-      <c r="T3" s="20">
+      <c r="T3" s="21">
         <v>0.0</v>
       </c>
-      <c r="U3" s="20">
+      <c r="U3" s="21">
         <v>0.0</v>
       </c>
-      <c r="V3" s="20">
+      <c r="V3" s="21">
         <v>0.0</v>
       </c>
-      <c r="W3" s="20">
+      <c r="W3" s="21">
         <v>0.0</v>
       </c>
-      <c r="X3" s="20">
+      <c r="X3" s="21">
         <v>930.0</v>
       </c>
     </row>
     <row r="4" ht="18.0" customHeight="1">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="19">
+      <c r="C4" s="20">
         <v>143.0</v>
       </c>
-      <c r="D4" s="19" t="s">
-        <v>316</v>
-      </c>
-      <c r="E4" s="19">
+      <c r="D4" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="E4" s="20">
         <v>1.0</v>
       </c>
-      <c r="F4" s="19">
+      <c r="F4" s="20">
         <v>0.0</v>
       </c>
-      <c r="G4" s="19">
+      <c r="G4" s="20">
         <v>0.0</v>
       </c>
-      <c r="H4" s="19">
+      <c r="H4" s="20">
         <v>1.0</v>
       </c>
-      <c r="I4" s="20">
+      <c r="I4" s="21">
         <v>0.0</v>
       </c>
-      <c r="J4" s="20">
+      <c r="J4" s="21">
         <v>0.0</v>
       </c>
-      <c r="K4" s="20">
+      <c r="K4" s="21">
         <v>2.0</v>
       </c>
-      <c r="L4" s="20">
+      <c r="L4" s="21">
         <v>0.0</v>
       </c>
-      <c r="M4" s="20">
+      <c r="M4" s="21">
         <v>1.0</v>
       </c>
-      <c r="N4" s="20">
+      <c r="N4" s="21">
         <v>0.0</v>
       </c>
-      <c r="O4" s="20">
+      <c r="O4" s="21">
         <v>0.0</v>
       </c>
-      <c r="P4" s="20">
+      <c r="P4" s="21">
         <v>0.0</v>
       </c>
-      <c r="Q4" s="20">
+      <c r="Q4" s="21">
         <v>0.0</v>
       </c>
-      <c r="R4" s="20">
+      <c r="R4" s="21">
         <v>1.0</v>
       </c>
-      <c r="S4" s="20">
+      <c r="S4" s="21">
         <v>0.0</v>
       </c>
-      <c r="T4" s="20">
+      <c r="T4" s="21">
         <v>0.0</v>
       </c>
-      <c r="U4" s="20">
+      <c r="U4" s="21">
         <v>0.0</v>
       </c>
-      <c r="V4" s="20">
+      <c r="V4" s="21">
         <v>0.0</v>
       </c>
-      <c r="W4" s="20">
+      <c r="W4" s="21">
         <v>0.0</v>
       </c>
-      <c r="X4" s="20">
+      <c r="X4" s="21">
         <v>940.0</v>
       </c>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="20">
         <v>144.0</v>
       </c>
-      <c r="D5" s="19" t="s">
-        <v>317</v>
-      </c>
-      <c r="E5" s="19">
+      <c r="D5" s="20" t="s">
+        <v>319</v>
+      </c>
+      <c r="E5" s="20">
         <v>1.0</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="20">
         <v>0.0</v>
       </c>
-      <c r="G5" s="19">
+      <c r="G5" s="20">
         <v>0.0</v>
       </c>
-      <c r="H5" s="19">
+      <c r="H5" s="20">
         <v>1.0</v>
       </c>
-      <c r="I5" s="20">
+      <c r="I5" s="21">
         <v>0.0</v>
       </c>
-      <c r="J5" s="20">
+      <c r="J5" s="21">
         <v>0.0</v>
       </c>
-      <c r="K5" s="20">
+      <c r="K5" s="21">
         <v>2.0</v>
       </c>
-      <c r="L5" s="20">
+      <c r="L5" s="21">
         <v>0.0</v>
       </c>
-      <c r="M5" s="20">
+      <c r="M5" s="21">
         <v>1.0</v>
       </c>
-      <c r="N5" s="20">
+      <c r="N5" s="21">
         <v>0.0</v>
       </c>
-      <c r="O5" s="20">
+      <c r="O5" s="21">
         <v>0.0</v>
       </c>
-      <c r="P5" s="20">
+      <c r="P5" s="21">
         <v>0.0</v>
       </c>
-      <c r="Q5" s="20">
+      <c r="Q5" s="21">
         <v>0.0</v>
       </c>
-      <c r="R5" s="20">
+      <c r="R5" s="21">
         <v>1.0</v>
       </c>
-      <c r="S5" s="20">
+      <c r="S5" s="21">
         <v>0.0</v>
       </c>
-      <c r="T5" s="20">
+      <c r="T5" s="21">
         <v>0.0</v>
       </c>
-      <c r="U5" s="20">
+      <c r="U5" s="21">
         <v>0.0</v>
       </c>
-      <c r="V5" s="20">
+      <c r="V5" s="21">
         <v>0.0</v>
       </c>
-      <c r="W5" s="20">
+      <c r="W5" s="21">
         <v>0.0</v>
       </c>
-      <c r="X5" s="20">
+      <c r="X5" s="21">
         <v>950.0</v>
       </c>
     </row>
     <row r="6" ht="36.0" customHeight="1">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="20">
         <v>145.0</v>
       </c>
-      <c r="D6" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="E6" s="19">
+      <c r="D6" s="19" t="s">
+        <v>320</v>
+      </c>
+      <c r="E6" s="20">
         <v>1.0</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="20">
         <v>0.0</v>
       </c>
-      <c r="G6" s="19">
+      <c r="G6" s="20">
         <v>0.0</v>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="20">
         <v>1.0</v>
       </c>
-      <c r="I6" s="20">
+      <c r="I6" s="21">
         <v>0.0</v>
       </c>
-      <c r="J6" s="20">
+      <c r="J6" s="21">
         <v>0.0</v>
       </c>
-      <c r="K6" s="20">
+      <c r="K6" s="21">
         <v>2.0</v>
       </c>
-      <c r="L6" s="20">
+      <c r="L6" s="21">
         <v>0.0</v>
       </c>
-      <c r="M6" s="20">
+      <c r="M6" s="21">
         <v>1.0</v>
       </c>
-      <c r="N6" s="20">
+      <c r="N6" s="21">
         <v>0.0</v>
       </c>
-      <c r="O6" s="20">
+      <c r="O6" s="21">
         <v>0.0</v>
       </c>
-      <c r="P6" s="20">
+      <c r="P6" s="21">
         <v>0.0</v>
       </c>
-      <c r="Q6" s="20">
+      <c r="Q6" s="21">
         <v>0.0</v>
       </c>
-      <c r="R6" s="20">
+      <c r="R6" s="21">
         <v>1.0</v>
       </c>
-      <c r="S6" s="20">
+      <c r="S6" s="21">
         <v>0.0</v>
       </c>
-      <c r="T6" s="20">
+      <c r="T6" s="21">
         <v>0.0</v>
       </c>
-      <c r="U6" s="20">
+      <c r="U6" s="21">
         <v>0.0</v>
       </c>
-      <c r="V6" s="20">
+      <c r="V6" s="21">
         <v>0.0</v>
       </c>
-      <c r="W6" s="20">
+      <c r="W6" s="21">
         <v>0.0</v>
       </c>
-      <c r="X6" s="20">
+      <c r="X6" s="21">
         <v>960.0</v>
       </c>
     </row>
@@ -7021,13 +7040,13 @@
   <sheetData>
     <row r="1" ht="24.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -7038,13 +7057,13 @@
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="3" ht="18.0" customHeight="1">
@@ -7058,7 +7077,7 @@
         <v>12</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" ht="18.0" customHeight="1">
@@ -7066,13 +7085,13 @@
         <v>22</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="5" ht="18.0" customHeight="1">
@@ -7080,13 +7099,13 @@
         <v>25</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="6" ht="18.0" customHeight="1">
@@ -7094,13 +7113,13 @@
         <v>28</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="7" ht="18.0" customHeight="1">
@@ -7111,10 +7130,10 @@
         <v>199</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="8" ht="18.0" customHeight="1">
@@ -7122,13 +7141,13 @@
         <v>35</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>31</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="9" ht="18.0" customHeight="1">
@@ -7136,13 +7155,13 @@
         <v>35</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="10" ht="18.0" customHeight="1">
@@ -7150,13 +7169,13 @@
         <v>39</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="11" ht="18.0" customHeight="1">
@@ -7164,13 +7183,13 @@
         <v>39</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="12" ht="36.0" customHeight="1">
@@ -7178,13 +7197,13 @@
         <v>43</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>31</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="13" ht="36.0" customHeight="1">
@@ -7192,13 +7211,13 @@
         <v>49</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>39</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1"/>
@@ -15312,7 +15331,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" ht="18.0" customHeight="1">
+    <row r="4" ht="30.0" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -15340,11 +15359,11 @@
       <c r="I4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="J4" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>100</v>
+      <c r="J4" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>212</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>70</v>
@@ -15358,19 +15377,19 @@
         <v>13</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>124</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>95</v>
@@ -15382,13 +15401,13 @@
         <v>70</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="6" ht="18.0" customHeight="1">
+    <row r="6" ht="30.75" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -15396,13 +15415,13 @@
         <v>13</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>67</v>
@@ -15420,13 +15439,13 @@
         <v>81</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="7" ht="18.0" customHeight="1">
+    <row r="7" ht="35.25" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
@@ -15434,13 +15453,13 @@
         <v>13</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>67</v>
@@ -15458,7 +15477,7 @@
         <v>81</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>70</v>
@@ -15472,13 +15491,13 @@
         <v>13</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>67</v>
@@ -15496,7 +15515,7 @@
         <v>81</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>70</v>
@@ -15510,13 +15529,13 @@
         <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>67</v>
@@ -15534,7 +15553,7 @@
         <v>81</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>70</v>
@@ -16609,13 +16628,13 @@
         <v>40</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>124</v>
@@ -16636,7 +16655,7 @@
         <v>127</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" ht="18.0" customHeight="1">
@@ -16685,13 +16704,13 @@
         <v>40</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>124</v>
@@ -16709,7 +16728,7 @@
         <v>70</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>70</v>
@@ -16723,13 +16742,13 @@
         <v>40</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>67</v>
@@ -16747,7 +16766,7 @@
         <v>70</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>70</v>
@@ -16761,19 +16780,19 @@
         <v>40</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>124</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>95</v>
@@ -16785,7 +16804,7 @@
         <v>70</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>70</v>
@@ -16799,19 +16818,19 @@
         <v>40</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>124</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>95</v>
@@ -16823,7 +16842,7 @@
         <v>70</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>70</v>
@@ -16837,13 +16856,13 @@
         <v>40</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>124</v>
@@ -16899,7 +16918,7 @@
         <v>151</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>70</v>
@@ -16945,16 +16964,16 @@
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="E11" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>95</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1"/>
@@ -17009,7 +17028,11 @@
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1"/>
     <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
+    <row r="21" ht="14.25" customHeight="1">
+      <c r="E21" s="8" t="s">
+        <v>260</v>
+      </c>
+    </row>
     <row r="22" ht="14.25" customHeight="1"/>
     <row r="23" ht="14.25" customHeight="1"/>
     <row r="24" ht="14.25" customHeight="1"/>
@@ -18061,13 +18084,13 @@
         <v>32</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>124</v>
@@ -18088,7 +18111,7 @@
         <v>127</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3" ht="18.0" customHeight="1">
@@ -18140,7 +18163,7 @@
         <v>197</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>199</v>
@@ -18161,7 +18184,7 @@
         <v>70</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>70</v>
@@ -18175,19 +18198,19 @@
         <v>32</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>124</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>69</v>
@@ -18199,7 +18222,7 @@
         <v>70</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>70</v>
@@ -18213,19 +18236,19 @@
         <v>32</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>67</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>95</v>
@@ -18233,11 +18256,11 @@
       <c r="I6" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J6" s="12">
         <v>0.0</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>70</v>
@@ -18321,16 +18344,16 @@
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="E9" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>95</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1"/>

</xml_diff>